<commit_message>
ADD: new price from 09.03.2026
</commit_message>
<xml_diff>
--- a/data/cards.xlsx
+++ b/data/cards.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sveto\OneDrive\Desktop\eko_inv\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E2E85F8-FC82-4672-A79A-D2C6B10BB9D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22AF96AB-5AAA-4DC8-9BCA-8870FDE7181F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2617,13 +2617,13 @@
     <t>Демакс АД % Група 2</t>
   </si>
   <si>
-    <t>Демакс ди пи ай % група 1</t>
-  </si>
-  <si>
-    <t>Демакс ди пи ай % група 2</t>
-  </si>
-  <si>
-    <t>Демакс ди пи ай % група 3</t>
+    <t>Демакс Ди Пи Ай % група 3</t>
+  </si>
+  <si>
+    <t>Демакс Ди Пи Ай % група 2</t>
+  </si>
+  <si>
+    <t>Демакс Ди Пи Ай % група 1</t>
   </si>
 </sst>
 </file>
@@ -7117,7 +7117,7 @@
     </row>
     <row r="377" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A377" t="s">
-        <v>865</v>
+        <v>867</v>
       </c>
       <c r="B377" t="s">
         <v>788</v>
@@ -7161,7 +7161,7 @@
     </row>
     <row r="381" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A381" t="s">
-        <v>867</v>
+        <v>865</v>
       </c>
       <c r="B381" t="s">
         <v>796</v>

</xml_diff>

<commit_message>
ADD: new prices from 20.03.2026
</commit_message>
<xml_diff>
--- a/data/cards.xlsx
+++ b/data/cards.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sveto\OneDrive\Desktop\eko_inv\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sveto\OneDrive\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64A58F50-755E-40FF-858D-3634E974C45F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{214E020B-7CF4-4E67-8F99-D311052A4A60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1295" uniqueCount="903">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1295" uniqueCount="904">
   <si>
     <t>Company</t>
   </si>
@@ -2729,6 +2729,9 @@
   </si>
   <si>
     <t>СВ1180ХР</t>
+  </si>
+  <si>
+    <t>78970151027720864</t>
   </si>
 </sst>
 </file>
@@ -2790,7 +2793,7 @@
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -7512,7 +7515,7 @@
         <v>820</v>
       </c>
       <c r="C401" s="1" t="s">
-        <v>814</v>
+        <v>903</v>
       </c>
     </row>
     <row r="402" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
UPDATE: card from Rubin went to Euroway
</commit_message>
<xml_diff>
--- a/data/cards.xlsx
+++ b/data/cards.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sveto\OneDrive\Desktop\eko_inv\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6E04D60-6DDF-43FB-85E3-50D659461BDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43A26C22-5C48-4B1A-8E9D-917E3BDE22AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1376" uniqueCount="956">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1376" uniqueCount="954">
   <si>
     <t>Company</t>
   </si>
@@ -2870,12 +2870,6 @@
   </si>
   <si>
     <t>6</t>
-  </si>
-  <si>
-    <t>РУБИН АД</t>
-  </si>
-  <si>
-    <t>Р2</t>
   </si>
   <si>
     <t>78970153027721009</t>
@@ -3395,7 +3389,7 @@
         <v>26</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>953</v>
+        <v>951</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -8053,13 +8047,13 @@
     </row>
     <row r="437" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A437" t="s">
+        <v>903</v>
+      </c>
+      <c r="B437" s="1" t="s">
+        <v>907</v>
+      </c>
+      <c r="C437" s="2" t="s">
         <v>950</v>
-      </c>
-      <c r="B437" t="s">
-        <v>951</v>
-      </c>
-      <c r="C437" s="2" t="s">
-        <v>952</v>
       </c>
     </row>
     <row r="438" spans="1:4" x14ac:dyDescent="0.25">
@@ -8292,10 +8286,10 @@
         <v>946</v>
       </c>
       <c r="C456" s="2" t="s">
-        <v>954</v>
+        <v>952</v>
       </c>
       <c r="D456" t="s">
-        <v>955</v>
+        <v>953</v>
       </c>
     </row>
   </sheetData>

</xml_diff>